<commit_message>
Add North Carolina auto and home insurance: 13 verified facts
Lean pass: auto minimums (50/100/50, raised July 2025 from 30/60/25,
cross-confirmed by both NCDOI and NC DMV), mandatory UM/UIM, FS-1 proof
of insurance, and lapse penalties. Home: NC's FAIR Plan and Coastal
Property Insurance Pool (Beach Plan), from the plans' own administrator
site. NC already had correct numbers in a Secondary-unverified
placeholder; upgraded to Primary source rather than duplicating.

README updated via the safe manual-shift method (no insert_rows).
Verified: integrity_check, foreign_key_check, exact fact-card counts
(7 auto, 6 home) in the built pages. 84/84 tests pass, 34 pages build.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA/Insurance_Reference_Data_v5.xlsx
+++ b/DATA/Insurance_Reference_Data_v5.xlsx
@@ -34,6 +34,8 @@
     <sheet name="PA Home Verified" sheetId="25" state="visible" r:id="rId25"/>
     <sheet name="GA Auto Verified" sheetId="26" state="visible" r:id="rId26"/>
     <sheet name="GA Home Verified" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="NC Auto Verified" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="NC Home Verified" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CA Auto Verified'!$A$1:$L$32</definedName>
@@ -703,7 +705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="28" min="1" max="1"/>
@@ -725,7 +727,7 @@
       </c>
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>Structured reference data from research through October 1, 2026 (California auto and home; Texas, Florida, New York, Illinois, Pennsylvania and Georgia auto; Texas, Florida, New York, Illinois, Pennsylvania and Georgia home verified from primary sources; California home credit-use rules still open) for the U.S. auto and home insurance education/comparison project.</t>
+          <t>Structured reference data from research through October 1, 2026 (California auto and home; Texas, Florida, New York, Illinois, Pennsylvania, Georgia and North Carolina auto; Texas, Florida, New York, Illinois, Pennsylvania, Georgia and North Carolina home verified from primary sources; California home credit-use rules still open) for the U.S. auto and home insurance education/comparison project.</t>
         </is>
       </c>
     </row>
@@ -1419,19 +1421,19 @@
         <f>COUNTIF('GA Home Verified'!$J$2:$J$500,"Primary source")</f>
         <v/>
       </c>
-      <c r="C37">
+      <c r="C37" s="28">
         <f>COUNTIF('GA Home Verified'!$J$2:$J$500,"Secondary - unverified")</f>
         <v/>
       </c>
-      <c r="D37">
+      <c r="D37" s="28">
         <f>COUNTIF('GA Home Verified'!$J$2:$J$500,"Conflicting")</f>
         <v/>
       </c>
-      <c r="E37">
+      <c r="E37" s="28">
         <f>COUNTIF('GA Home Verified'!$J$2:$J$500,"Not researched")</f>
         <v/>
       </c>
-      <c r="F37">
+      <c r="F37" s="28">
         <f>SUM(B37:E37)</f>
         <v/>
       </c>
@@ -1439,347 +1441,425 @@
     <row r="38" ht="15" customHeight="1" s="29">
       <c r="A38" s="39" t="inlineStr">
         <is>
-          <t>All tabs</t>
+          <t>NC Auto Verified</t>
         </is>
       </c>
       <c r="B38" s="39">
-        <f>SUM(B17:B37)</f>
+        <f>COUNTIF('NC Auto Verified'!$J$2:$J$500,"Primary source")</f>
         <v/>
       </c>
-      <c r="C38">
-        <f>SUM(C17:C37)</f>
+      <c r="C38" s="28">
+        <f>COUNTIF('NC Auto Verified'!$J$2:$J$500,"Secondary - unverified")</f>
         <v/>
       </c>
-      <c r="D38">
-        <f>SUM(D17:D37)</f>
+      <c r="D38" s="28">
+        <f>COUNTIF('NC Auto Verified'!$J$2:$J$500,"Conflicting")</f>
         <v/>
       </c>
-      <c r="E38">
-        <f>SUM(E17:E37)</f>
+      <c r="E38" s="28">
+        <f>COUNTIF('NC Auto Verified'!$J$2:$J$500,"Not researched")</f>
         <v/>
       </c>
-      <c r="F38">
-        <f>SUM(F17:F37)</f>
+      <c r="F38" s="28">
+        <f>SUM(B38:E38)</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="29">
       <c r="A39" s="39" t="inlineStr">
         <is>
-          <t>TX Home Verified</t>
-        </is>
-      </c>
-      <c r="B39" s="39" t="inlineStr">
-        <is>
-          <t>Texas home facts from TDI, TWIA and secondary sources.</t>
-        </is>
+          <t>NC Home Verified</t>
+        </is>
+      </c>
+      <c r="B39" s="39">
+        <f>COUNTIF('NC Home Verified'!$J$2:$J$500,"Primary source")</f>
+        <v/>
+      </c>
+      <c r="C39">
+        <f>COUNTIF('NC Home Verified'!$J$2:$J$500,"Secondary - unverified")</f>
+        <v/>
+      </c>
+      <c r="D39">
+        <f>COUNTIF('NC Home Verified'!$J$2:$J$500,"Conflicting")</f>
+        <v/>
+      </c>
+      <c r="E39">
+        <f>COUNTIF('NC Home Verified'!$J$2:$J$500,"Not researched")</f>
+        <v/>
+      </c>
+      <c r="F39">
+        <f>SUM(B39:E39)</f>
+        <v/>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="29">
       <c r="A40" s="39" t="inlineStr">
         <is>
-          <t>FL Home Verified</t>
-        </is>
-      </c>
-      <c r="B40" s="39" t="inlineStr">
-        <is>
-          <t>Florida home facts: hurricane deductibles, Citizens and flood rules.</t>
-        </is>
+          <t>All tabs</t>
+        </is>
+      </c>
+      <c r="B40" s="39">
+        <f>SUM(B17:B39)</f>
+        <v/>
+      </c>
+      <c r="C40">
+        <f>SUM(C17:C39)</f>
+        <v/>
+      </c>
+      <c r="D40">
+        <f>SUM(D17:D39)</f>
+        <v/>
+      </c>
+      <c r="E40">
+        <f>SUM(E17:E39)</f>
+        <v/>
+      </c>
+      <c r="F40">
+        <f>SUM(F17:F39)</f>
+        <v/>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="29">
       <c r="A41" s="39" t="inlineStr">
         <is>
-          <t>TX Auto Verified</t>
+          <t>TX Home Verified</t>
         </is>
       </c>
       <c r="B41" s="39" t="inlineStr">
         <is>
-          <t>Texas auto facts from the TDI guide.</t>
+          <t>Texas home facts from TDI, TWIA and secondary sources.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="29">
       <c r="A42" s="39" t="inlineStr">
         <is>
-          <t>FL Auto Verified</t>
+          <t>FL Home Verified</t>
         </is>
       </c>
       <c r="B42" s="39" t="inlineStr">
         <is>
-          <t>Florida auto facts from FLHSMV and Florida Statutes.</t>
+          <t>Florida home facts: hurricane deductibles, Citizens and flood rules.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="29">
       <c r="A43" s="39" t="inlineStr">
         <is>
-          <t>NY Auto Verified</t>
+          <t>TX Auto Verified</t>
         </is>
       </c>
       <c r="B43" s="39" t="inlineStr">
         <is>
-          <t>New York auto facts from the DFS consumer guide.</t>
+          <t>Texas auto facts from the TDI guide.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="29">
       <c r="A44" s="39" t="inlineStr">
         <is>
-          <t>CA Home Verified</t>
+          <t>FL Auto Verified</t>
         </is>
       </c>
       <c r="B44" s="39" t="inlineStr">
         <is>
-          <t>California home insurance facts traced to CDI, CEA and FAIR Plan sources and CDI press releases.</t>
+          <t>Florida auto facts from FLHSMV and Florida Statutes.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="29">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>CA Auto Verified</t>
+          <t>NY Auto Verified</t>
         </is>
       </c>
       <c r="B45" s="39" t="inlineStr">
         <is>
-          <t>California auto facts traced to primary sources (CDI, DMV, statutes and regulations).</t>
+          <t>New York auto facts from the DFS consumer guide.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="29">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>State Min Limits</t>
+          <t>CA Home Verified</t>
         </is>
       </c>
       <c r="B46" s="39" t="inlineStr">
         <is>
-          <t>Minimum auto liability limits by state (50 states + DC); most rows still to research.</t>
+          <t>California home insurance facts traced to CDI, CEA and FAIR Plan sources and CDI press releases.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="29">
       <c r="A47" s="39" t="inlineStr">
         <is>
-          <t>Rating Factors</t>
+          <t>CA Auto Verified</t>
         </is>
       </c>
       <c r="B47" s="39" t="inlineStr">
         <is>
-          <t>Credit, gender and age rules by state for states researched.</t>
+          <t>California auto facts traced to primary sources (CDI, DMV, statutes and regulations).</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="29">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>Discounts</t>
+          <t>State Min Limits</t>
         </is>
       </c>
       <c r="B48" s="39" t="inlineStr">
         <is>
-          <t>Discount availability by state and carrier.</t>
+          <t>Minimum auto liability limits by state (50 states + DC); most rows still to research.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="29">
       <c r="A49" s="39" t="inlineStr">
         <is>
-          <t>Telematics</t>
+          <t>Rating Factors</t>
         </is>
       </c>
       <c r="B49" s="39" t="inlineStr">
         <is>
-          <t>Usage-based programs by carrier.</t>
+          <t>Credit, gender and age rules by state for states researched.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="29">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>Coverage Details</t>
+          <t>Discounts</t>
         </is>
       </c>
       <c r="B50" s="39" t="inlineStr">
         <is>
-          <t>Flood, earthquake, umbrella and other coverage facts.</t>
+          <t>Discount availability by state and carrier.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="29">
       <c r="A51" s="39" t="inlineStr">
         <is>
-          <t>Price Benchmarks</t>
+          <t>Telematics</t>
         </is>
       </c>
       <c r="B51" s="39" t="inlineStr">
         <is>
-          <t>Published average premiums with spread formulas.</t>
+          <t>Usage-based programs by carrier.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="29">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>Regulatory Watch</t>
+          <t>Coverage Details</t>
         </is>
       </c>
       <c r="B52" s="39" t="inlineStr">
         <is>
-          <t>Laws and rules to monitor.</t>
+          <t>Flood, earthquake, umbrella and other coverage facts.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="39" t="inlineStr">
         <is>
-          <t>Quote Source Options</t>
+          <t>Price Benchmarks</t>
         </is>
       </c>
       <c r="B53" s="39" t="inlineStr">
         <is>
-          <t>Ways to get real quotes and what each implies.</t>
+          <t>Published average premiums with spread formulas.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="39" t="inlineStr">
         <is>
-          <t>Legal Review Checklist</t>
+          <t>Regulatory Watch</t>
         </is>
       </c>
       <c r="B54" s="39" t="inlineStr">
         <is>
-          <t>Questions to bring to insurance-regulatory counsel.</t>
+          <t>Laws and rules to monitor.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>Refresh Schedule</t>
+          <t>Quote Source Options</t>
         </is>
       </c>
       <c r="B55" s="39" t="inlineStr">
         <is>
-          <t>Owners, review intervals and overdue checks (formulas).</t>
+          <t>Ways to get real quotes and what each implies.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="28" t="inlineStr">
         <is>
-          <t>Conflicts Log</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Where sources disagree and what to verify.</t>
+          <t>Legal Review Checklist</t>
+        </is>
+      </c>
+      <c r="B56" s="28" t="inlineStr">
+        <is>
+          <t>Questions to bring to insurance-regulatory counsel.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="28" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Refresh Schedule</t>
         </is>
       </c>
       <c r="B57" s="28" t="inlineStr">
         <is>
-          <t>Every source used, with type and reliability note.</t>
+          <t>Owners, review intervals and overdue checks (formulas).</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="28" t="inlineStr">
         <is>
-          <t>Tabs (additional entries below)</t>
-        </is>
-      </c>
-      <c r="B58" s="28" t="n"/>
+          <t>Conflicts Log</t>
+        </is>
+      </c>
+      <c r="B58" s="28" t="inlineStr">
+        <is>
+          <t>Where sources disagree and what to verify.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="28" t="inlineStr">
         <is>
-          <t>NY Home Verified</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B59" s="28" t="inlineStr">
         <is>
-          <t>New York home facts from the DFS homeowners guide, NYPIUA, and the cancellations/non-renewals and discounts pages.</t>
+          <t>Every source used, with type and reliability note.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="28" t="inlineStr">
         <is>
-          <t>IL Auto Verified</t>
-        </is>
-      </c>
-      <c r="B60" s="28" t="inlineStr">
-        <is>
-          <t>Illinois auto facts from the IDOI shopping guide and the Illinois credit-scoring statute.</t>
-        </is>
-      </c>
+          <t>Tabs (additional entries below)</t>
+        </is>
+      </c>
+      <c r="B60" s="28" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="28" t="inlineStr">
         <is>
+          <t>NY Home Verified</t>
+        </is>
+      </c>
+      <c r="B61" s="28" t="inlineStr">
+        <is>
+          <t>New York home facts from the DFS homeowners guide, NYPIUA, and the cancellations/non-renewals and discounts pages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="28" t="inlineStr">
+        <is>
+          <t>IL Auto Verified</t>
+        </is>
+      </c>
+      <c r="B62" s="28" t="inlineStr">
+        <is>
+          <t>Illinois auto facts from the IDOI shopping guide and the Illinois credit-scoring statute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="28" t="inlineStr">
+        <is>
           <t>IL Home Verified</t>
         </is>
       </c>
-      <c r="B61" s="28" t="inlineStr">
+      <c r="B63" s="28" t="inlineStr">
         <is>
           <t>Illinois home facts from the IDOI homeowner guide, the Illinois FAIR Plan, non-renewal rules, and the credit-scoring statute.</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="28" t="inlineStr">
         <is>
           <t>PA Auto Verified</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B64" s="28" t="inlineStr">
         <is>
           <t>Pennsylvania auto facts from the official IDOI Automobile Insurance Guide.</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="28" t="inlineStr">
         <is>
           <t>PA Home Verified</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B65" s="28" t="inlineStr">
         <is>
           <t>Pennsylvania home facts from the official IDOI Homeowners Insurance Guide and the PA FAIR Plan.</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>GA Auto Verified</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B66" t="inlineStr">
         <is>
           <t>Georgia auto facts from the official OCI Consumer Guide for Automobile Insurance.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>GA Home Verified</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Georgia home facts from the official OCI Consumer Guide for Homeowners Insurance and the Georgia FAIR Plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>NC Auto Verified</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>North Carolina auto facts from NCDOI and the NC DMV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>NC Home Verified</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>North Carolina home facts from the NCJUA/NCIUA FAIR and Beach Plans.</t>
         </is>
       </c>
     </row>
@@ -1790,19 +1870,19 @@
     <mergeCell ref="B54:F54"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B46:F46"/>
+    <mergeCell ref="B56:F56"/>
     <mergeCell ref="B52:F52"/>
+    <mergeCell ref="B12:F12"/>
     <mergeCell ref="B43:F43"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B39:F39"/>
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B42:F42"/>
     <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B53:F53"/>
     <mergeCell ref="B44:F44"/>
-    <mergeCell ref="B53:F53"/>
     <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B40:F40"/>
     <mergeCell ref="B49:F49"/>
+    <mergeCell ref="B55:F55"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B51:F51"/>
@@ -13360,7 +13440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E112"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="58" customWidth="1" style="28" min="1" max="1"/>
@@ -16034,6 +16114,81 @@
         </is>
       </c>
       <c r="E109" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI - Changes to the Rating of Automobile Insurance Policies</t>
+        </is>
+      </c>
+      <c r="B110" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C110" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdoi.gov/changes-rating-automobile-insurance-policies-effective-july-1-2025</t>
+        </is>
+      </c>
+      <c r="D110" s="28" t="inlineStr">
+        <is>
+          <t>Official NCDOI bulletin page.</t>
+        </is>
+      </c>
+      <c r="E110" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="28" t="inlineStr">
+        <is>
+          <t>NC DMV - Vehicle Insurance Requirements</t>
+        </is>
+      </c>
+      <c r="B111" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C111" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdot.gov/dmv/title-registration/insurance-requirements/Pages/default.aspx</t>
+        </is>
+      </c>
+      <c r="D111" s="28" t="inlineStr">
+        <is>
+          <t>Official NCDOT DMV consumer page; cross-confirms NCDOI's numbers.</t>
+        </is>
+      </c>
+      <c r="E111" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="28" t="inlineStr">
+        <is>
+          <t>NC Joint Underwriting Association / Insurance Underwriting Association (FAIR/Beach Plans)</t>
+        </is>
+      </c>
+      <c r="B112" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C112" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncjua-nciua.org/html/svcs_cov.htm</t>
+        </is>
+      </c>
+      <c r="D112" s="28" t="inlineStr">
+        <is>
+          <t>Official site of the plans' own administrator.</t>
+        </is>
+      </c>
+      <c r="E112" s="48" t="n">
         <v>46296</v>
       </c>
     </row>
@@ -22692,6 +22847,847 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Legal Citation</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>Date Collected</t>
+        </is>
+      </c>
+      <c r="H1" s="28" t="inlineStr">
+        <is>
+          <t>Geographic Scope</t>
+        </is>
+      </c>
+      <c r="I1" s="28" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="J1" s="28" t="inlineStr">
+        <is>
+          <t>Verification Status</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>Bodily injury per person</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>$50,000 (raised from $30,000 for policies issued/renewed on or after July 1, 2025)</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI bulletin</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI - Changes to the Rating of Automobile Insurance Policies</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdoi.gov/changes-rating-automobile-insurance-policies-effective-july-1-2025</t>
+        </is>
+      </c>
+      <c r="G2" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K2" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Bodily injury per accident</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>$100,000 (raised from $60,000 for policies issued/renewed on or after July 1, 2025)</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI bulletin</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI - Changes to the Rating of Automobile Insurance Policies</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdoi.gov/changes-rating-automobile-insurance-policies-effective-july-1-2025</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J3" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K3" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Property damage</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>$50,000 (raised from $25,000 for policies issued/renewed on or after July 1, 2025)</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI bulletin</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI - Changes to the Rating of Automobile Insurance Policies</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdoi.gov/changes-rating-automobile-insurance-policies-effective-july-1-2025</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Underinsured motorist now required</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Underinsured motorist coverage is included in all new or renewed policies on or after July 1, 2025; previously, policies at the old minimum limits did not include it automatically</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI bulletin</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>NCDOI - Changes to the Rating of Automobile Insurance Policies</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdoi.gov/changes-rating-automobile-insurance-policies-effective-july-1-2025</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Uninsured motorist coverage</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>Uninsured/underinsured motorist coverage is mandated on all policies, even those exceeding the minimum liability limits</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>NC DMV insurance requirements page</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>NC DMV - Vehicle Insurance Requirements</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdot.gov/dmv/title-registration/insurance-requirements/Pages/default.aspx</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Proof of insurance (FS-1)</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Insurance companies must electronically submit a Certificate of Insurance (FS-1) to demonstrate continuous coverage; only policies from insurers licensed to do business in North Carolina are accepted, so out-of-state policies are rejected</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>NC DMV insurance requirements page</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>NC DMV - Vehicle Insurance Requirements</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdot.gov/dmv/title-registration/insurance-requirements/Pages/default.aspx</t>
+        </is>
+      </c>
+      <c r="G7" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I7" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J7" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K7" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>Cancellation</t>
+        </is>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Penalties for a lapse in coverage</t>
+        </is>
+      </c>
+      <c r="C8" s="28" t="inlineStr">
+        <is>
+          <t>Civil penalties for a lapse range from $50 to $150 depending on prior lapse history within three years, plus a $50 restoration fee at registration renewal; license plate revocation is possible for unpaid penalties</t>
+        </is>
+      </c>
+      <c r="D8" s="28" t="inlineStr">
+        <is>
+          <t>NC DMV insurance requirements page</t>
+        </is>
+      </c>
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>NC DMV - Vehicle Insurance Requirements</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncdot.gov/dmv/title-registration/insurance-requirements/Pages/default.aspx</t>
+        </is>
+      </c>
+      <c r="G8" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H8" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I8" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J8" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K8" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Legal Citation</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>Date Collected</t>
+        </is>
+      </c>
+      <c r="H1" s="28" t="inlineStr">
+        <is>
+          <t>Geographic Scope</t>
+        </is>
+      </c>
+      <c r="I1" s="28" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="J1" s="28" t="inlineStr">
+        <is>
+          <t>Verification Status</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>NC FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>A market of last resort created by the NC General Assembly in 1969, offering full peril commercial fire and dwelling fire coverage statewide, excluding the beach area</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>NCJUA/NCIUA (FAIR/Beach Plans administrator)</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>NC Joint Underwriting Association / Insurance Underwriting Association (FAIR/Beach Plans)</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncjua-nciua.org/html/svcs_cov.htm</t>
+        </is>
+      </c>
+      <c r="G2" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K2" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>NC FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Coverage limits</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Maximum residential building coverage of $1,000,000; personal property capped at 40% of the building coverage limit</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>NCJUA/NCIUA (FAIR/Beach Plans administrator)</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>NC Joint Underwriting Association / Insurance Underwriting Association (FAIR/Beach Plans)</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncjua-nciua.org/html/svcs_cov.htm</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J3" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K3" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>NC Beach Plan</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>The Coastal Property Insurance Pool (formerly the Beach Plan) offers commercial, homeowner, and dwelling windstorm coverage, plus homeowner and commercial fire coverage, to properties in the 18 eligible coastal counties</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>NCJUA/NCIUA (FAIR/Beach Plans administrator)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>NC Joint Underwriting Association / Insurance Underwriting Association (FAIR/Beach Plans)</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncjua-nciua.org/html/svcs_cov.htm</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>NC Beach Plan</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Coverage limits</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Maximum residential building coverage of $1,000,000; personal property capped at 40% of the building coverage limit; maximum commercial combined limit of $4 million</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>NCJUA/NCIUA (FAIR/Beach Plans administrator)</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>NC Joint Underwriting Association / Insurance Underwriting Association (FAIR/Beach Plans)</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncjua-nciua.org/html/svcs_cov.htm</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>NC Beach Plan</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Windstorm eligibility condition</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>The windstorm product requires an active primary coverage policy from a carrier admitted in North Carolina that has excluded windstorm coverage</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>NCJUA/NCIUA (FAIR/Beach Plans administrator)</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>NC Joint Underwriting Association / Insurance Underwriting Association (FAIR/Beach Plans)</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncjua-nciua.org/html/svcs_cov.htm</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>NC FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Market of last resort</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>Both the FAIR Plan and the Coastal Property Insurance Pool are a market of last resort; applicants are expected to attempt to obtain insurance in the standard market first</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>NCJUA/NCIUA (FAIR/Beach Plans administrator)</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>NC Joint Underwriting Association / Insurance Underwriting Association (FAIR/Beach Plans)</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>https://www.ncjua-nciua.org/html/svcs_cov.htm</t>
+        </is>
+      </c>
+      <c r="G7" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="I7" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J7" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K7" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -32163,24 +33159,28 @@
       </c>
       <c r="E35" s="41" t="n"/>
       <c r="F35" s="41" t="n"/>
-      <c r="G35" s="41" t="n"/>
+      <c r="G35" s="41" t="inlineStr">
+        <is>
+          <t>UM/UIM mandated on all policies</t>
+        </is>
+      </c>
       <c r="H35" s="41" t="inlineStr">
         <is>
-          <t>Raised in 2025 per source</t>
+          <t>Raised from 30/60/25, effective for policies issued/renewed on or after July 1, 2025</t>
         </is>
       </c>
       <c r="I35" s="41" t="inlineStr">
         <is>
-          <t>CarInsurance.com - Minimum liability by state (Apr 2026)</t>
+          <t>NCDOI - Changes to the Rating of Automobile Insurance Policies</t>
         </is>
       </c>
       <c r="J35" s="42" t="inlineStr">
         <is>
-          <t>https://www.carinsurance.com/Articles/minimum-liability-car-insurance-requirements-by-state.aspx</t>
+          <t>https://www.ncdoi.gov/changes-rating-automobile-insurance-policies-effective-july-1-2025</t>
         </is>
       </c>
       <c r="K35" s="43" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L35" s="41" t="inlineStr">
         <is>
@@ -32189,16 +33189,16 @@
       </c>
       <c r="M35" s="41" t="inlineStr">
         <is>
-          <t>Reference data (secondary source)</t>
+          <t>Regulator-published</t>
         </is>
       </c>
       <c r="N35" s="45" t="inlineStr">
         <is>
-          <t>Secondary - unverified</t>
+          <t>Primary source</t>
         </is>
       </c>
       <c r="O35" s="43" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="P35" s="41" t="n"/>
     </row>

</xml_diff>

<commit_message>
Add Washington auto and home insurance data (first-time research, no conflict)
Auto: WA OIC's own mandatory insurance law page confirms the 25/50/10
minimum liability, alternatives to carrying insurance (certificate of
deposit, $60,000 surety bond, or self-insurance for 26+ vehicles), and
the proof-of-insurance ticket requirement.

Home: the Washington FAIR Plan's own FAQ page (established 1968, a
Joint Reinsurance Association funded entirely by member insurers, no
taxpayer money) - basic fire coverage only, excludes liability, theft
and most water damage.

5 new auto facts, 6 new home facts, 2 new sources, 1 new min_limit row
(Washington had no prior data or logged conflict), all Primary source.
Database: 118 sources, 323 rule_fact rows, 306/323 from regulator/
government sources, 14 open conflicts (unchanged - none were logged
for Washington).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA/Insurance_Reference_Data_v5.xlsx
+++ b/DATA/Insurance_Reference_Data_v5.xlsx
@@ -40,6 +40,8 @@
     <sheet name="NJ Home Verified" sheetId="31" state="visible" r:id="rId31"/>
     <sheet name="VA Auto Verified" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="VA Home Verified" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="WA Auto Verified" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="WA Home Verified" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CA Auto Verified'!$A$1:$L$32</definedName>
@@ -709,7 +711,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F77"/>
+  <dimension ref="A1:F81"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="28" min="1" max="1"/>
@@ -732,7 +734,7 @@
       </c>
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>Structured reference data from research through October 1, 2026 (California auto and home; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey and Virginia auto; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey and Virginia home verified from primary sources; California home credit-use rules still open) for the U.S. auto and home insurance education/comparison project.</t>
+          <t>Structured reference data from research through October 1, 2026 (California auto and home; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey, Virginia and Washington auto; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey, Virginia and Washington home verified from primary sources; California home credit-use rules still open) for the U.S. auto and home insurance education/comparison project.</t>
         </is>
       </c>
     </row>
@@ -1590,19 +1592,19 @@
         <f>COUNTIF('VA Home Verified'!$J$2:$J$500,"Primary source")</f>
         <v/>
       </c>
-      <c r="C43">
+      <c r="C43" s="28">
         <f>COUNTIF('VA Home Verified'!$J$2:$J$500,"Secondary - unverified")</f>
         <v/>
       </c>
-      <c r="D43">
+      <c r="D43" s="28">
         <f>COUNTIF('VA Home Verified'!$J$2:$J$500,"Conflicting")</f>
         <v/>
       </c>
-      <c r="E43">
+      <c r="E43" s="28">
         <f>COUNTIF('VA Home Verified'!$J$2:$J$500,"Not researched")</f>
         <v/>
       </c>
-      <c r="F43">
+      <c r="F43" s="28">
         <f>SUM(B43:E43)</f>
         <v/>
       </c>
@@ -1610,286 +1612,316 @@
     <row r="44" ht="15" customHeight="1" s="29">
       <c r="A44" s="39" t="inlineStr">
         <is>
-          <t>All tabs</t>
+          <t>WA Auto Verified</t>
         </is>
       </c>
       <c r="B44" s="39">
-        <f>SUM(B17:B43)</f>
+        <f>COUNTIF('WA Auto Verified'!$J$2:$J$500,"Primary source")</f>
         <v/>
       </c>
-      <c r="C44">
-        <f>SUM(C17:C43)</f>
+      <c r="C44" s="28">
+        <f>COUNTIF('WA Auto Verified'!$J$2:$J$500,"Secondary - unverified")</f>
         <v/>
       </c>
-      <c r="D44">
-        <f>SUM(D17:D43)</f>
+      <c r="D44" s="28">
+        <f>COUNTIF('WA Auto Verified'!$J$2:$J$500,"Conflicting")</f>
         <v/>
       </c>
-      <c r="E44">
-        <f>SUM(E17:E43)</f>
+      <c r="E44" s="28">
+        <f>COUNTIF('WA Auto Verified'!$J$2:$J$500,"Not researched")</f>
         <v/>
       </c>
-      <c r="F44">
-        <f>SUM(F17:F43)</f>
+      <c r="F44" s="28">
+        <f>SUM(B44:E44)</f>
         <v/>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="29">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>TX Home Verified</t>
-        </is>
-      </c>
-      <c r="B45" s="39" t="inlineStr">
-        <is>
-          <t>Texas home facts from TDI, TWIA and secondary sources.</t>
-        </is>
+          <t>WA Home Verified</t>
+        </is>
+      </c>
+      <c r="B45" s="39">
+        <f>COUNTIF('WA Home Verified'!$J$2:$J$500,"Primary source")</f>
+        <v/>
+      </c>
+      <c r="C45">
+        <f>COUNTIF('WA Home Verified'!$J$2:$J$500,"Secondary - unverified")</f>
+        <v/>
+      </c>
+      <c r="D45">
+        <f>COUNTIF('WA Home Verified'!$J$2:$J$500,"Conflicting")</f>
+        <v/>
+      </c>
+      <c r="E45">
+        <f>COUNTIF('WA Home Verified'!$J$2:$J$500,"Not researched")</f>
+        <v/>
+      </c>
+      <c r="F45">
+        <f>SUM(B45:E45)</f>
+        <v/>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="29">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>FL Home Verified</t>
-        </is>
-      </c>
-      <c r="B46" s="39" t="inlineStr">
-        <is>
-          <t>Florida home facts: hurricane deductibles, Citizens and flood rules.</t>
-        </is>
+          <t>All tabs</t>
+        </is>
+      </c>
+      <c r="B46" s="39">
+        <f>SUM(B17:B45)</f>
+        <v/>
+      </c>
+      <c r="C46">
+        <f>SUM(C17:C45)</f>
+        <v/>
+      </c>
+      <c r="D46">
+        <f>SUM(D17:D45)</f>
+        <v/>
+      </c>
+      <c r="E46">
+        <f>SUM(E17:E45)</f>
+        <v/>
+      </c>
+      <c r="F46">
+        <f>SUM(F17:F45)</f>
+        <v/>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="29">
       <c r="A47" s="39" t="inlineStr">
         <is>
-          <t>TX Auto Verified</t>
+          <t>TX Home Verified</t>
         </is>
       </c>
       <c r="B47" s="39" t="inlineStr">
         <is>
-          <t>Texas auto facts from the TDI guide.</t>
+          <t>Texas home facts from TDI, TWIA and secondary sources.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="29">
       <c r="A48" s="39" t="inlineStr">
         <is>
-          <t>FL Auto Verified</t>
+          <t>FL Home Verified</t>
         </is>
       </c>
       <c r="B48" s="39" t="inlineStr">
         <is>
-          <t>Florida auto facts from FLHSMV and Florida Statutes.</t>
+          <t>Florida home facts: hurricane deductibles, Citizens and flood rules.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="29">
       <c r="A49" s="39" t="inlineStr">
         <is>
-          <t>NY Auto Verified</t>
+          <t>TX Auto Verified</t>
         </is>
       </c>
       <c r="B49" s="39" t="inlineStr">
         <is>
-          <t>New York auto facts from the DFS consumer guide.</t>
+          <t>Texas auto facts from the TDI guide.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="29">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>CA Home Verified</t>
+          <t>FL Auto Verified</t>
         </is>
       </c>
       <c r="B50" s="39" t="inlineStr">
         <is>
-          <t>California home insurance facts traced to CDI, CEA and FAIR Plan sources and CDI press releases.</t>
+          <t>Florida auto facts from FLHSMV and Florida Statutes.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="29">
       <c r="A51" s="39" t="inlineStr">
         <is>
-          <t>CA Auto Verified</t>
+          <t>NY Auto Verified</t>
         </is>
       </c>
       <c r="B51" s="39" t="inlineStr">
         <is>
-          <t>California auto facts traced to primary sources (CDI, DMV, statutes and regulations).</t>
+          <t>New York auto facts from the DFS consumer guide.</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="29">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>State Min Limits</t>
+          <t>CA Home Verified</t>
         </is>
       </c>
       <c r="B52" s="39" t="inlineStr">
         <is>
-          <t>Minimum auto liability limits by state (50 states + DC); most rows still to research.</t>
+          <t>California home insurance facts traced to CDI, CEA and FAIR Plan sources and CDI press releases.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="39" t="inlineStr">
         <is>
-          <t>Rating Factors</t>
+          <t>CA Auto Verified</t>
         </is>
       </c>
       <c r="B53" s="39" t="inlineStr">
         <is>
-          <t>Credit, gender and age rules by state for states researched.</t>
+          <t>California auto facts traced to primary sources (CDI, DMV, statutes and regulations).</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="39" t="inlineStr">
         <is>
-          <t>Discounts</t>
+          <t>State Min Limits</t>
         </is>
       </c>
       <c r="B54" s="39" t="inlineStr">
         <is>
-          <t>Discount availability by state and carrier.</t>
+          <t>Minimum auto liability limits by state (50 states + DC); most rows still to research.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>Telematics</t>
+          <t>Rating Factors</t>
         </is>
       </c>
       <c r="B55" s="39" t="inlineStr">
         <is>
-          <t>Usage-based programs by carrier.</t>
+          <t>Credit, gender and age rules by state for states researched.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="28" t="inlineStr">
         <is>
-          <t>Coverage Details</t>
+          <t>Discounts</t>
         </is>
       </c>
       <c r="B56" s="28" t="inlineStr">
         <is>
-          <t>Flood, earthquake, umbrella and other coverage facts.</t>
+          <t>Discount availability by state and carrier.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="28" t="inlineStr">
         <is>
-          <t>Price Benchmarks</t>
+          <t>Telematics</t>
         </is>
       </c>
       <c r="B57" s="28" t="inlineStr">
         <is>
-          <t>Published average premiums with spread formulas.</t>
+          <t>Usage-based programs by carrier.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="28" t="inlineStr">
         <is>
-          <t>Regulatory Watch</t>
+          <t>Coverage Details</t>
         </is>
       </c>
       <c r="B58" s="28" t="inlineStr">
         <is>
-          <t>Laws and rules to monitor.</t>
+          <t>Flood, earthquake, umbrella and other coverage facts.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="28" t="inlineStr">
         <is>
-          <t>Quote Source Options</t>
+          <t>Price Benchmarks</t>
         </is>
       </c>
       <c r="B59" s="28" t="inlineStr">
         <is>
-          <t>Ways to get real quotes and what each implies.</t>
+          <t>Published average premiums with spread formulas.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="28" t="inlineStr">
         <is>
-          <t>Legal Review Checklist</t>
+          <t>Regulatory Watch</t>
         </is>
       </c>
       <c r="B60" s="28" t="inlineStr">
         <is>
-          <t>Questions to bring to insurance-regulatory counsel.</t>
+          <t>Laws and rules to monitor.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="28" t="inlineStr">
         <is>
-          <t>Refresh Schedule</t>
+          <t>Quote Source Options</t>
         </is>
       </c>
       <c r="B61" s="28" t="inlineStr">
         <is>
-          <t>Owners, review intervals and overdue checks (formulas).</t>
+          <t>Ways to get real quotes and what each implies.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="28" t="inlineStr">
         <is>
-          <t>Conflicts Log</t>
+          <t>Legal Review Checklist</t>
         </is>
       </c>
       <c r="B62" s="28" t="inlineStr">
         <is>
-          <t>Where sources disagree and what to verify.</t>
+          <t>Questions to bring to insurance-regulatory counsel.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="28" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Refresh Schedule</t>
         </is>
       </c>
       <c r="B63" s="28" t="inlineStr">
         <is>
-          <t>Every source used, with type and reliability note.</t>
+          <t>Owners, review intervals and overdue checks (formulas).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="28" t="inlineStr">
         <is>
-          <t>Tabs (additional entries below)</t>
+          <t>Conflicts Log</t>
         </is>
       </c>
       <c r="B64" s="28" t="inlineStr">
         <is>
-          <t>Illinois auto facts from the IDOI shopping guide and the Illinois credit-scoring statute.</t>
+          <t>Where sources disagree and what to verify.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="28" t="inlineStr">
         <is>
-          <t>NY Home Verified</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B65" s="28" t="inlineStr">
         <is>
-          <t>New York home facts from the DFS homeowners guide, NYPIUA, and the cancellations/non-renewals and discounts pages.</t>
+          <t>Every source used, with type and reliability note.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="28" t="inlineStr">
         <is>
-          <t>IL Auto Verified</t>
+          <t>Tabs (additional entries below)</t>
         </is>
       </c>
       <c r="B66" s="28" t="inlineStr">
@@ -1901,132 +1933,180 @@
     <row r="67">
       <c r="A67" s="28" t="inlineStr">
         <is>
-          <t>IL Home Verified</t>
+          <t>NY Home Verified</t>
         </is>
       </c>
       <c r="B67" s="28" t="inlineStr">
         <is>
-          <t>Illinois home facts from the IDOI homeowner guide, the Illinois FAIR Plan, non-renewal rules, and the credit-scoring statute.</t>
+          <t>New York home facts from the DFS homeowners guide, NYPIUA, and the cancellations/non-renewals and discounts pages.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="28" t="inlineStr">
         <is>
-          <t>PA Auto Verified</t>
+          <t>IL Auto Verified</t>
         </is>
       </c>
       <c r="B68" s="28" t="inlineStr">
         <is>
-          <t>Pennsylvania auto facts from the official IDOI Automobile Insurance Guide.</t>
+          <t>Illinois auto facts from the IDOI shopping guide and the Illinois credit-scoring statute.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="28" t="inlineStr">
         <is>
-          <t>PA Home Verified</t>
+          <t>IL Home Verified</t>
         </is>
       </c>
       <c r="B69" s="28" t="inlineStr">
         <is>
-          <t>Pennsylvania home facts from the official IDOI Homeowners Insurance Guide and the PA FAIR Plan.</t>
+          <t>Illinois home facts from the IDOI homeowner guide, the Illinois FAIR Plan, non-renewal rules, and the credit-scoring statute.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="28" t="inlineStr">
         <is>
-          <t>GA Auto Verified</t>
+          <t>PA Auto Verified</t>
         </is>
       </c>
       <c r="B70" s="28" t="inlineStr">
         <is>
-          <t>Georgia auto facts from the official OCI Consumer Guide for Automobile Insurance.</t>
+          <t>Pennsylvania auto facts from the official IDOI Automobile Insurance Guide.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="28" t="inlineStr">
         <is>
-          <t>GA Home Verified</t>
+          <t>PA Home Verified</t>
         </is>
       </c>
       <c r="B71" s="28" t="inlineStr">
         <is>
-          <t>Georgia home facts from the official OCI Consumer Guide for Homeowners Insurance and the Georgia FAIR Plan.</t>
+          <t>Pennsylvania home facts from the official IDOI Homeowners Insurance Guide and the PA FAIR Plan.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="28" t="inlineStr">
         <is>
-          <t>NC Auto Verified</t>
+          <t>GA Auto Verified</t>
         </is>
       </c>
       <c r="B72" s="28" t="inlineStr">
         <is>
-          <t>North Carolina auto facts from NCDOI and the NC DMV.</t>
+          <t>Georgia auto facts from the official OCI Consumer Guide for Automobile Insurance.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="28" t="inlineStr">
         <is>
+          <t>GA Home Verified</t>
+        </is>
+      </c>
+      <c r="B73" s="28" t="inlineStr">
+        <is>
+          <t>Georgia home facts from the official OCI Consumer Guide for Homeowners Insurance and the Georgia FAIR Plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="28" t="inlineStr">
+        <is>
+          <t>NC Auto Verified</t>
+        </is>
+      </c>
+      <c r="B74" s="28" t="inlineStr">
+        <is>
+          <t>North Carolina auto facts from NCDOI and the NC DMV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="28" t="inlineStr">
+        <is>
           <t>NC Home Verified</t>
         </is>
       </c>
-      <c r="B73" s="28" t="inlineStr">
+      <c r="B75" s="28" t="inlineStr">
         <is>
           <t>North Carolina home facts from the NCJUA/NCIUA FAIR and Beach Plans.</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="28" t="inlineStr">
         <is>
           <t>NJ Auto Verified</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
+      <c r="B76" s="28" t="inlineStr">
         <is>
           <t>New Jersey auto facts from the NJDOBI bulletin on 2026 minimum-limit increases and the verbatim AICRA statute (N.J.S.A. 39:6A-3.1) for the Basic Policy.</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="28" t="inlineStr">
         <is>
           <t>NJ Home Verified</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B77" s="28" t="inlineStr">
         <is>
           <t>New Jersey home facts from the official NJDOBI consumer guide and the NJIUA (FAIR Plan).</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>VA Auto Verified</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B78" t="inlineStr">
         <is>
           <t>Virginia auto facts from the official VA DMV insurance-requirements page.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
+    <row r="79">
+      <c r="A79" t="inlineStr">
         <is>
           <t>VA Home Verified</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Virginia home facts from the Virginia Property Insurance Association (VPIA / FAIR Plan).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>WA Auto Verified</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Washington auto facts from the official WA OIC mandatory insurance law page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>WA Home Verified</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Washington home facts from the Washington FAIR Plan's own FAQ page.</t>
         </is>
       </c>
     </row>
@@ -2035,9 +2115,9 @@
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="B47:F47"/>
     <mergeCell ref="B54:F54"/>
+    <mergeCell ref="B62:F62"/>
     <mergeCell ref="B3:F3"/>
     <mergeCell ref="B59:F59"/>
-    <mergeCell ref="B46:F46"/>
     <mergeCell ref="B58:F58"/>
     <mergeCell ref="B56:F56"/>
     <mergeCell ref="B52:F52"/>
@@ -2045,6 +2125,7 @@
     <mergeCell ref="B48:F48"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B60:F60"/>
+    <mergeCell ref="B61:F61"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B53:F53"/>
@@ -2054,7 +2135,6 @@
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B51:F51"/>
-    <mergeCell ref="B45:F45"/>
     <mergeCell ref="B50:F50"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -13615,7 +13695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="58" customWidth="1" style="28" min="1" max="1"/>
@@ -16489,6 +16569,56 @@
         </is>
       </c>
       <c r="E117" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="28" t="inlineStr">
+        <is>
+          <t>Washington OIC - Mandatory Auto/Motorcycle Insurance Law</t>
+        </is>
+      </c>
+      <c r="B118" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C118" s="28" t="inlineStr">
+        <is>
+          <t>https://www.insurance.wa.gov/washington-states-mandatory-automotorcycle-insurance-law</t>
+        </is>
+      </c>
+      <c r="D118" s="28" t="inlineStr">
+        <is>
+          <t>Official Washington OIC consumer page, read directly.</t>
+        </is>
+      </c>
+      <c r="E118" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan - Frequently Asked Questions</t>
+        </is>
+      </c>
+      <c r="B119" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C119" s="28" t="inlineStr">
+        <is>
+          <t>https://www.wafairplan.com/faq/</t>
+        </is>
+      </c>
+      <c r="D119" s="28" t="inlineStr">
+        <is>
+          <t>Official site of the plan's own administrator (Washington's FAIR Plan).</t>
+        </is>
+      </c>
+      <c r="E119" s="48" t="n">
         <v>46296</v>
       </c>
     </row>
@@ -28485,6 +28615,741 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Legal Citation</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>Date Collected</t>
+        </is>
+      </c>
+      <c r="H1" s="28" t="inlineStr">
+        <is>
+          <t>Geographic Scope</t>
+        </is>
+      </c>
+      <c r="I1" s="28" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="J1" s="28" t="inlineStr">
+        <is>
+          <t>Verification Status</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>Bodily injury per person</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>$25,000</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>WA OIC mandatory insurance law page (25/50/10)</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Washington OIC - Mandatory Auto/Motorcycle Insurance Law</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>https://www.insurance.wa.gov/washington-states-mandatory-automotorcycle-insurance-law</t>
+        </is>
+      </c>
+      <c r="G2" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K2" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Bodily injury per accident</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>$50,000</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>WA OIC mandatory insurance law page (25/50/10)</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>Washington OIC - Mandatory Auto/Motorcycle Insurance Law</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>https://www.insurance.wa.gov/washington-states-mandatory-automotorcycle-insurance-law</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J3" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K3" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Property damage</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>$10,000</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>WA OIC mandatory insurance law page (25/50/10)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Washington OIC - Mandatory Auto/Motorcycle Insurance Law</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>https://www.insurance.wa.gov/washington-states-mandatory-automotorcycle-insurance-law</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Alternatives to carrying insurance</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Instead of liability insurance, a driver may file a certificate of deposit with the Department of Licensing, or a liability bond of at least $60,000 from an authorized surety bond company; self-insurance is available only to those with 26 or more vehicles</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>WA OIC mandatory insurance law page</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>Washington OIC - Mandatory Auto/Motorcycle Insurance Law</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>https://www.insurance.wa.gov/washington-states-mandatory-automotorcycle-insurance-law</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Cancellation</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Proof-of-insurance requirement</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>If stopped by a law enforcement officer, a driver must show proof of auto/motorcycle insurance; failure to do so results in a traffic violation ticket</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>WA OIC mandatory insurance law page</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Washington OIC - Mandatory Auto/Motorcycle Insurance Law</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>https://www.insurance.wa.gov/washington-states-mandatory-automotorcycle-insurance-law</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Legal Citation</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>Date Collected</t>
+        </is>
+      </c>
+      <c r="H1" s="28" t="inlineStr">
+        <is>
+          <t>Geographic Scope</t>
+        </is>
+      </c>
+      <c r="I1" s="28" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="J1" s="28" t="inlineStr">
+        <is>
+          <t>Verification Status</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>The Washington FAIR ('Fair Access to Insurance Requirements') Plan was established in 1968 to provide basic property insurance to applicants who cannot obtain property insurance in the standard insurance market; it is a Joint Reinsurance Association, with every insurer licensed to write property insurance in the state required to be a member, and receives no taxpayer or state funding</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>WA FAIR Plan FAQ (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan - Frequently Asked Questions</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>https://www.wafairplan.com/faq/</t>
+        </is>
+      </c>
+      <c r="G2" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K2" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Coverage provided</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Basic fire insurance for owner- and tenant-occupied dwellings, apartment buildings, commercial structures, and personal property/contents; Extended Coverage and Vandalism coverage are available</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>WA FAIR Plan FAQ (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan - Frequently Asked Questions</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>https://www.wafairplan.com/faq/</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J3" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K3" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Exclusions</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Coverage for liability, theft, and most types of water-related losses is not available through the Plan</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>WA FAIR Plan FAQ (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan - Frequently Asked Questions</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>https://www.wafairplan.com/faq/</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Eligibility</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>A last-resort option limited to applicants who are unable to obtain property coverage in the standard insurance market</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>WA FAIR Plan FAQ (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan - Frequently Asked Questions</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>https://www.wafairplan.com/faq/</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Deductibles</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>A range of deductibles is available, similar to standard-market policies</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>WA FAIR Plan FAQ (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan - Frequently Asked Questions</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>https://www.wafairplan.com/faq/</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="C7" s="28" t="inlineStr">
+        <is>
+          <t>2122 164th Street SW, Suite 301, Lynnwood, WA 98087; (425) 745-9808 or (866) 745-9808; wafairplan@wafairplan.com</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>WA FAIR Plan FAQ (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>Washington FAIR Plan - Frequently Asked Questions</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="inlineStr">
+        <is>
+          <t>https://www.wafairplan.com/faq/</t>
+        </is>
+      </c>
+      <c r="G7" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H7" s="28" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="I7" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J7" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K7" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -36066,17 +36931,31 @@
           <t>Washington</t>
         </is>
       </c>
-      <c r="B49" s="41" t="n"/>
-      <c r="C49" s="41" t="n"/>
-      <c r="D49" s="41" t="n"/>
+      <c r="B49" s="41" t="n">
+        <v>25</v>
+      </c>
+      <c r="C49" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="D49" s="41" t="n">
+        <v>10</v>
+      </c>
       <c r="E49" s="41" t="n"/>
       <c r="F49" s="41" t="n"/>
       <c r="G49" s="41" t="n"/>
       <c r="H49" s="41" t="n"/>
-      <c r="I49" s="41" t="n"/>
-      <c r="J49" s="42" t="n"/>
+      <c r="I49" s="41" t="inlineStr">
+        <is>
+          <t>Washington OIC - Mandatory Auto/Motorcycle Insurance Law</t>
+        </is>
+      </c>
+      <c r="J49" s="42" t="inlineStr">
+        <is>
+          <t>https://www.insurance.wa.gov/washington-states-mandatory-automotorcycle-insurance-law</t>
+        </is>
+      </c>
       <c r="K49" s="43" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L49" s="41" t="inlineStr">
         <is>
@@ -36085,16 +36964,16 @@
       </c>
       <c r="M49" s="41" t="inlineStr">
         <is>
-          <t>Placeholder</t>
+          <t>Regulator-published</t>
         </is>
       </c>
       <c r="N49" s="47" t="inlineStr">
         <is>
-          <t>Not researched</t>
+          <t>Primary source</t>
         </is>
       </c>
       <c r="O49" s="43" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="P49" s="41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Indiana auto and home insurance data (first-time research, no conflict)
Indiana's own legislature site (iga.in.gov) renders its code pages via
JavaScript and could not be read directly, so facts are sourced from the
verbatim Indiana Code text via a legal-code aggregator.

Auto: Indiana Code 9-25-4-5 confirms the 25/50/25 minimum (property
damage raised from $10,000 effective July 1, 2018); Indiana Code
27-7-5-2 adds the UM/UIM availability and rejection rules, including the
$50,000 floor on underinsured motorist coverage.

Home: the Indiana FAIR Plan (established 1968, a true market of last
resort) read directly from its own website - 3-declination eligibility,
dwelling/commercial coverage, and the $250,000/$1,000,000 coverage caps.

5 new auto facts, 5 new home facts, 3 new sources, 1 new min_limit row,
all Primary source. Database: 131 sources, 350 rule_fact rows, 333/350
from regulator/government sources.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DATA/Insurance_Reference_Data_v5.xlsx
+++ b/DATA/Insurance_Reference_Data_v5.xlsx
@@ -46,6 +46,8 @@
     <sheet name="AZ Home Verified" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="TN Auto Verified" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="TN Home Verified" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="IN Auto Verified" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="IN Home Verified" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'CA Auto Verified'!$A$1:$L$32</definedName>
@@ -715,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F89"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="28" min="1" max="1"/>
@@ -738,7 +740,7 @@
       </c>
       <c r="B3" s="32" t="inlineStr">
         <is>
-          <t>Structured reference data from research through October 1, 2026 (California auto and home; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey, Virginia, Washington, Arizona and Tennessee auto; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey, Virginia, Washington, Arizona and Tennessee home verified from primary sources; California home credit-use rules still open) for the U.S. auto and home insurance education/comparison project.</t>
+          <t>Structured reference data from research through October 1, 2026 (California auto and home; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey, Virginia, Washington, Arizona, Tennessee and Indiana auto; Texas, Florida, New York, Illinois, Pennsylvania, Georgia, North Carolina, New Jersey, Virginia, Washington, Arizona, Tennessee and Indiana home verified from primary sources; California home credit-use rules still open) for the U.S. auto and home insurance education/comparison project.</t>
         </is>
       </c>
     </row>
@@ -1758,19 +1760,19 @@
         <f>COUNTIF('TN Home Verified'!$J$2:$J$500,"Primary source")</f>
         <v/>
       </c>
-      <c r="C49">
+      <c r="C49" s="28">
         <f>COUNTIF('TN Home Verified'!$J$2:$J$500,"Secondary - unverified")</f>
         <v/>
       </c>
-      <c r="D49">
+      <c r="D49" s="28">
         <f>COUNTIF('TN Home Verified'!$J$2:$J$500,"Conflicting")</f>
         <v/>
       </c>
-      <c r="E49">
+      <c r="E49" s="28">
         <f>COUNTIF('TN Home Verified'!$J$2:$J$500,"Not researched")</f>
         <v/>
       </c>
-      <c r="F49">
+      <c r="F49" s="28">
         <f>SUM(B49:E49)</f>
         <v/>
       </c>
@@ -1778,286 +1780,316 @@
     <row r="50" ht="15" customHeight="1" s="29">
       <c r="A50" s="39" t="inlineStr">
         <is>
-          <t>All tabs</t>
+          <t>IN Auto Verified</t>
         </is>
       </c>
       <c r="B50" s="39">
-        <f>SUM(B17:B49)</f>
+        <f>COUNTIF('IN Auto Verified'!$J$2:$J$500,"Primary source")</f>
         <v/>
       </c>
-      <c r="C50">
-        <f>SUM(C17:C49)</f>
+      <c r="C50" s="28">
+        <f>COUNTIF('IN Auto Verified'!$J$2:$J$500,"Secondary - unverified")</f>
         <v/>
       </c>
-      <c r="D50">
-        <f>SUM(D17:D49)</f>
+      <c r="D50" s="28">
+        <f>COUNTIF('IN Auto Verified'!$J$2:$J$500,"Conflicting")</f>
         <v/>
       </c>
-      <c r="E50">
-        <f>SUM(E17:E49)</f>
+      <c r="E50" s="28">
+        <f>COUNTIF('IN Auto Verified'!$J$2:$J$500,"Not researched")</f>
         <v/>
       </c>
-      <c r="F50">
-        <f>SUM(F17:F49)</f>
+      <c r="F50" s="28">
+        <f>SUM(B50:E50)</f>
         <v/>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="29">
       <c r="A51" s="39" t="inlineStr">
         <is>
-          <t>TX Home Verified</t>
-        </is>
-      </c>
-      <c r="B51" s="39" t="inlineStr">
-        <is>
-          <t>Texas home facts from TDI, TWIA and secondary sources.</t>
-        </is>
+          <t>IN Home Verified</t>
+        </is>
+      </c>
+      <c r="B51" s="39">
+        <f>COUNTIF('IN Home Verified'!$J$2:$J$500,"Primary source")</f>
+        <v/>
+      </c>
+      <c r="C51">
+        <f>COUNTIF('IN Home Verified'!$J$2:$J$500,"Secondary - unverified")</f>
+        <v/>
+      </c>
+      <c r="D51">
+        <f>COUNTIF('IN Home Verified'!$J$2:$J$500,"Conflicting")</f>
+        <v/>
+      </c>
+      <c r="E51">
+        <f>COUNTIF('IN Home Verified'!$J$2:$J$500,"Not researched")</f>
+        <v/>
+      </c>
+      <c r="F51">
+        <f>SUM(B51:E51)</f>
+        <v/>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="29">
       <c r="A52" s="39" t="inlineStr">
         <is>
-          <t>FL Home Verified</t>
-        </is>
-      </c>
-      <c r="B52" s="39" t="inlineStr">
-        <is>
-          <t>Florida home facts: hurricane deductibles, Citizens and flood rules.</t>
-        </is>
+          <t>All tabs</t>
+        </is>
+      </c>
+      <c r="B52" s="39">
+        <f>SUM(B17:B51)</f>
+        <v/>
+      </c>
+      <c r="C52">
+        <f>SUM(C17:C51)</f>
+        <v/>
+      </c>
+      <c r="D52">
+        <f>SUM(D17:D51)</f>
+        <v/>
+      </c>
+      <c r="E52">
+        <f>SUM(E17:E51)</f>
+        <v/>
+      </c>
+      <c r="F52">
+        <f>SUM(F17:F51)</f>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="39" t="inlineStr">
         <is>
-          <t>TX Auto Verified</t>
+          <t>TX Home Verified</t>
         </is>
       </c>
       <c r="B53" s="39" t="inlineStr">
         <is>
-          <t>Texas auto facts from the TDI guide.</t>
+          <t>Texas home facts from TDI, TWIA and secondary sources.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="39" t="inlineStr">
         <is>
-          <t>FL Auto Verified</t>
+          <t>FL Home Verified</t>
         </is>
       </c>
       <c r="B54" s="39" t="inlineStr">
         <is>
-          <t>Florida auto facts from FLHSMV and Florida Statutes.</t>
+          <t>Florida home facts: hurricane deductibles, Citizens and flood rules.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="39" t="inlineStr">
         <is>
-          <t>NY Auto Verified</t>
+          <t>TX Auto Verified</t>
         </is>
       </c>
       <c r="B55" s="39" t="inlineStr">
         <is>
-          <t>New York auto facts from the DFS consumer guide.</t>
+          <t>Texas auto facts from the TDI guide.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="28" t="inlineStr">
         <is>
-          <t>CA Home Verified</t>
+          <t>FL Auto Verified</t>
         </is>
       </c>
       <c r="B56" s="28" t="inlineStr">
         <is>
-          <t>California home insurance facts traced to CDI, CEA and FAIR Plan sources and CDI press releases.</t>
+          <t>Florida auto facts from FLHSMV and Florida Statutes.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="28" t="inlineStr">
         <is>
-          <t>CA Auto Verified</t>
+          <t>NY Auto Verified</t>
         </is>
       </c>
       <c r="B57" s="28" t="inlineStr">
         <is>
-          <t>California auto facts traced to primary sources (CDI, DMV, statutes and regulations).</t>
+          <t>New York auto facts from the DFS consumer guide.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="28" t="inlineStr">
         <is>
-          <t>State Min Limits</t>
+          <t>CA Home Verified</t>
         </is>
       </c>
       <c r="B58" s="28" t="inlineStr">
         <is>
-          <t>Minimum auto liability limits by state (50 states + DC); most rows still to research.</t>
+          <t>California home insurance facts traced to CDI, CEA and FAIR Plan sources and CDI press releases.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="28" t="inlineStr">
         <is>
-          <t>Rating Factors</t>
+          <t>CA Auto Verified</t>
         </is>
       </c>
       <c r="B59" s="28" t="inlineStr">
         <is>
-          <t>Credit, gender and age rules by state for states researched.</t>
+          <t>California auto facts traced to primary sources (CDI, DMV, statutes and regulations).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="28" t="inlineStr">
         <is>
-          <t>Discounts</t>
+          <t>State Min Limits</t>
         </is>
       </c>
       <c r="B60" s="28" t="inlineStr">
         <is>
-          <t>Discount availability by state and carrier.</t>
+          <t>Minimum auto liability limits by state (50 states + DC); most rows still to research.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="28" t="inlineStr">
         <is>
-          <t>Telematics</t>
+          <t>Rating Factors</t>
         </is>
       </c>
       <c r="B61" s="28" t="inlineStr">
         <is>
-          <t>Usage-based programs by carrier.</t>
+          <t>Credit, gender and age rules by state for states researched.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="28" t="inlineStr">
         <is>
-          <t>Coverage Details</t>
+          <t>Discounts</t>
         </is>
       </c>
       <c r="B62" s="28" t="inlineStr">
         <is>
-          <t>Flood, earthquake, umbrella and other coverage facts.</t>
+          <t>Discount availability by state and carrier.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="28" t="inlineStr">
         <is>
-          <t>Price Benchmarks</t>
+          <t>Telematics</t>
         </is>
       </c>
       <c r="B63" s="28" t="inlineStr">
         <is>
-          <t>Published average premiums with spread formulas.</t>
+          <t>Usage-based programs by carrier.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="28" t="inlineStr">
         <is>
-          <t>Regulatory Watch</t>
+          <t>Coverage Details</t>
         </is>
       </c>
       <c r="B64" s="28" t="inlineStr">
         <is>
-          <t>Laws and rules to monitor.</t>
+          <t>Flood, earthquake, umbrella and other coverage facts.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="28" t="inlineStr">
         <is>
-          <t>Quote Source Options</t>
+          <t>Price Benchmarks</t>
         </is>
       </c>
       <c r="B65" s="28" t="inlineStr">
         <is>
-          <t>Ways to get real quotes and what each implies.</t>
+          <t>Published average premiums with spread formulas.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="28" t="inlineStr">
         <is>
-          <t>Legal Review Checklist</t>
+          <t>Regulatory Watch</t>
         </is>
       </c>
       <c r="B66" s="28" t="inlineStr">
         <is>
-          <t>Questions to bring to insurance-regulatory counsel.</t>
+          <t>Laws and rules to monitor.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="28" t="inlineStr">
         <is>
-          <t>Refresh Schedule</t>
+          <t>Quote Source Options</t>
         </is>
       </c>
       <c r="B67" s="28" t="inlineStr">
         <is>
-          <t>Owners, review intervals and overdue checks (formulas).</t>
+          <t>Ways to get real quotes and what each implies.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="28" t="inlineStr">
         <is>
-          <t>Conflicts Log</t>
+          <t>Legal Review Checklist</t>
         </is>
       </c>
       <c r="B68" s="28" t="inlineStr">
         <is>
-          <t>Where sources disagree and what to verify.</t>
+          <t>Questions to bring to insurance-regulatory counsel.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="28" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Refresh Schedule</t>
         </is>
       </c>
       <c r="B69" s="28" t="inlineStr">
         <is>
-          <t>Every source used, with type and reliability note.</t>
+          <t>Owners, review intervals and overdue checks (formulas).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="28" t="inlineStr">
         <is>
-          <t>Tabs (additional entries below)</t>
+          <t>Conflicts Log</t>
         </is>
       </c>
       <c r="B70" s="28" t="inlineStr">
         <is>
-          <t>Illinois auto facts from the IDOI shopping guide and the Illinois credit-scoring statute.</t>
+          <t>Where sources disagree and what to verify.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="28" t="inlineStr">
         <is>
-          <t>NY Home Verified</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B71" s="28" t="inlineStr">
         <is>
-          <t>New York home facts from the DFS homeowners guide, NYPIUA, and the cancellations/non-renewals and discounts pages.</t>
+          <t>Every source used, with type and reliability note.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="28" t="inlineStr">
         <is>
-          <t>IL Auto Verified</t>
+          <t>Tabs (additional entries below)</t>
         </is>
       </c>
       <c r="B72" s="28" t="inlineStr">
@@ -2069,204 +2101,252 @@
     <row r="73">
       <c r="A73" s="28" t="inlineStr">
         <is>
-          <t>IL Home Verified</t>
+          <t>NY Home Verified</t>
         </is>
       </c>
       <c r="B73" s="28" t="inlineStr">
         <is>
-          <t>Illinois home facts from the IDOI homeowner guide, the Illinois FAIR Plan, non-renewal rules, and the credit-scoring statute.</t>
+          <t>New York home facts from the DFS homeowners guide, NYPIUA, and the cancellations/non-renewals and discounts pages.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="28" t="inlineStr">
         <is>
-          <t>PA Auto Verified</t>
+          <t>IL Auto Verified</t>
         </is>
       </c>
       <c r="B74" s="28" t="inlineStr">
         <is>
-          <t>Pennsylvania auto facts from the official IDOI Automobile Insurance Guide.</t>
+          <t>Illinois auto facts from the IDOI shopping guide and the Illinois credit-scoring statute.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="28" t="inlineStr">
         <is>
-          <t>PA Home Verified</t>
+          <t>IL Home Verified</t>
         </is>
       </c>
       <c r="B75" s="28" t="inlineStr">
         <is>
-          <t>Pennsylvania home facts from the official IDOI Homeowners Insurance Guide and the PA FAIR Plan.</t>
+          <t>Illinois home facts from the IDOI homeowner guide, the Illinois FAIR Plan, non-renewal rules, and the credit-scoring statute.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="28" t="inlineStr">
         <is>
-          <t>GA Auto Verified</t>
+          <t>PA Auto Verified</t>
         </is>
       </c>
       <c r="B76" s="28" t="inlineStr">
         <is>
-          <t>Georgia auto facts from the official OCI Consumer Guide for Automobile Insurance.</t>
+          <t>Pennsylvania auto facts from the official IDOI Automobile Insurance Guide.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="28" t="inlineStr">
         <is>
-          <t>GA Home Verified</t>
+          <t>PA Home Verified</t>
         </is>
       </c>
       <c r="B77" s="28" t="inlineStr">
         <is>
-          <t>Georgia home facts from the official OCI Consumer Guide for Homeowners Insurance and the Georgia FAIR Plan.</t>
+          <t>Pennsylvania home facts from the official IDOI Homeowners Insurance Guide and the PA FAIR Plan.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="28" t="inlineStr">
         <is>
-          <t>NC Auto Verified</t>
+          <t>GA Auto Verified</t>
         </is>
       </c>
       <c r="B78" s="28" t="inlineStr">
         <is>
-          <t>North Carolina auto facts from NCDOI and the NC DMV.</t>
+          <t>Georgia auto facts from the official OCI Consumer Guide for Automobile Insurance.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="28" t="inlineStr">
         <is>
-          <t>NC Home Verified</t>
+          <t>GA Home Verified</t>
         </is>
       </c>
       <c r="B79" s="28" t="inlineStr">
         <is>
-          <t>North Carolina home facts from the NCJUA/NCIUA FAIR and Beach Plans.</t>
+          <t>Georgia home facts from the official OCI Consumer Guide for Homeowners Insurance and the Georgia FAIR Plan.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="28" t="inlineStr">
         <is>
-          <t>NJ Auto Verified</t>
+          <t>NC Auto Verified</t>
         </is>
       </c>
       <c r="B80" s="28" t="inlineStr">
         <is>
-          <t>New Jersey auto facts from the NJDOBI bulletin on 2026 minimum-limit increases and the verbatim AICRA statute (N.J.S.A. 39:6A-3.1) for the Basic Policy.</t>
+          <t>North Carolina auto facts from NCDOI and the NC DMV.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="28" t="inlineStr">
         <is>
-          <t>NJ Home Verified</t>
+          <t>NC Home Verified</t>
         </is>
       </c>
       <c r="B81" s="28" t="inlineStr">
         <is>
-          <t>New Jersey home facts from the official NJDOBI consumer guide and the NJIUA (FAIR Plan).</t>
+          <t>North Carolina home facts from the NCJUA/NCIUA FAIR and Beach Plans.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="28" t="inlineStr">
         <is>
-          <t>VA Auto Verified</t>
+          <t>NJ Auto Verified</t>
         </is>
       </c>
       <c r="B82" s="28" t="inlineStr">
         <is>
-          <t>Virginia auto facts from the official VA DMV insurance-requirements page.</t>
+          <t>New Jersey auto facts from the NJDOBI bulletin on 2026 minimum-limit increases and the verbatim AICRA statute (N.J.S.A. 39:6A-3.1) for the Basic Policy.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="28" t="inlineStr">
         <is>
-          <t>VA Home Verified</t>
+          <t>NJ Home Verified</t>
         </is>
       </c>
       <c r="B83" s="28" t="inlineStr">
         <is>
-          <t>Virginia home facts from the Virginia Property Insurance Association (VPIA / FAIR Plan).</t>
+          <t>New Jersey home facts from the official NJDOBI consumer guide and the NJIUA (FAIR Plan).</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="28" t="inlineStr">
         <is>
-          <t>WA Auto Verified</t>
+          <t>VA Auto Verified</t>
         </is>
       </c>
       <c r="B84" s="28" t="inlineStr">
         <is>
-          <t>Washington auto facts from the official WA OIC mandatory insurance law page.</t>
+          <t>Virginia auto facts from the official VA DMV insurance-requirements page.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="28" t="inlineStr">
         <is>
+          <t>VA Home Verified</t>
+        </is>
+      </c>
+      <c r="B85" s="28" t="inlineStr">
+        <is>
+          <t>Virginia home facts from the Virginia Property Insurance Association (VPIA / FAIR Plan).</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="28" t="inlineStr">
+        <is>
+          <t>WA Auto Verified</t>
+        </is>
+      </c>
+      <c r="B86" s="28" t="inlineStr">
+        <is>
+          <t>Washington auto facts from the official WA OIC mandatory insurance law page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="28" t="inlineStr">
+        <is>
           <t>WA Home Verified</t>
         </is>
       </c>
-      <c r="B85" s="28" t="inlineStr">
+      <c r="B87" s="28" t="inlineStr">
         <is>
           <t>Washington home facts from the Washington FAIR Plan's own FAQ page.</t>
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="28" t="inlineStr">
         <is>
           <t>AZ Auto Verified</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B88" s="28" t="inlineStr">
         <is>
           <t>Arizona auto facts from A.R.S. Sections 28-4009 and 28-4135, read directly from azleg.gov.</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="28" t="inlineStr">
         <is>
           <t>AZ Home Verified</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B89" s="28" t="inlineStr">
         <is>
           <t>Arizona home facts from A.R.S. Sections 20-2202 and 20-1652 (no state FAIR Plan; cancellation/nonrenewal rules), read directly from azleg.gov.</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t>TN Auto Verified</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>Tennessee auto facts from Tenn. Code Ann. Sections 55-12-102, 56-7-1303 and 56-7-1304.</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t>TN Home Verified</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>Tennessee home facts: no state FAIR Plan (per NAIC), plus Tenn. Code Ann. Sections 56-7-113 and 56-7-114.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>IN Auto Verified</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Indiana auto facts from Indiana Code Sections 9-25-4-5 and 27-7-5-2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>IN Home Verified</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Indiana home facts from the Indiana FAIR Plan's own website.</t>
         </is>
       </c>
     </row>
@@ -2280,21 +2360,21 @@
     <mergeCell ref="B66:F66"/>
     <mergeCell ref="B58:F58"/>
     <mergeCell ref="B56:F56"/>
-    <mergeCell ref="B52:F52"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B60:F60"/>
+    <mergeCell ref="B67:F67"/>
     <mergeCell ref="B61:F61"/>
     <mergeCell ref="B13:F13"/>
     <mergeCell ref="B57:F57"/>
     <mergeCell ref="B53:F53"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B65:F65"/>
+    <mergeCell ref="B68:F68"/>
     <mergeCell ref="B55:F55"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B64:F64"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B51:F51"/>
     <mergeCell ref="B63:F63"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -13855,7 +13935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E129"/>
+  <dimension ref="A1:E132"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="58" customWidth="1" style="28" min="1" max="1"/>
@@ -17029,6 +17109,81 @@
         </is>
       </c>
       <c r="E129" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code 9-25-4-5 - Financial Responsibility Minimum Limits</t>
+        </is>
+      </c>
+      <c r="B130" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C130" s="28" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-9-motor-vehicles/in-code-sect-9-25-4-5.html</t>
+        </is>
+      </c>
+      <c r="D130" s="28" t="inlineStr">
+        <is>
+          <t>Verbatim statute text (Indiana Code), read via a legal-code aggregator (iga.in.gov is a JS-rendered page that could not be read directly).</t>
+        </is>
+      </c>
+      <c r="E130" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code 27-7-5-2 - Uninsured/Underinsured Motorist Coverage</t>
+        </is>
+      </c>
+      <c r="B131" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C131" s="28" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-27-insurance/in-code-sect-27-7-5-2.html</t>
+        </is>
+      </c>
+      <c r="D131" s="28" t="inlineStr">
+        <is>
+          <t>Verbatim statute text (Indiana Code), read via a legal-code aggregator.</t>
+        </is>
+      </c>
+      <c r="E131" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (Indiana Basic Property Insurance Underwriting Association)</t>
+        </is>
+      </c>
+      <c r="B132" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="C132" s="28" t="inlineStr">
+        <is>
+          <t>https://www.indianafairplan.com</t>
+        </is>
+      </c>
+      <c r="D132" s="28" t="inlineStr">
+        <is>
+          <t>Official site of the plan's own administrator (Indiana's FAIR Plan).</t>
+        </is>
+      </c>
+      <c r="E132" s="48" t="n">
         <v>46296</v>
       </c>
     </row>
@@ -32085,6 +32240,688 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Legal Citation</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>Date Collected</t>
+        </is>
+      </c>
+      <c r="H1" s="28" t="inlineStr">
+        <is>
+          <t>Geographic Scope</t>
+        </is>
+      </c>
+      <c r="I1" s="28" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="J1" s="28" t="inlineStr">
+        <is>
+          <t>Verification Status</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>Bodily injury per person</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>$25,000</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code Section 9-25-4-5</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code 9-25-4-5 - Financial Responsibility Minimum Limits</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-9-motor-vehicles/in-code-sect-9-25-4-5.html</t>
+        </is>
+      </c>
+      <c r="G2" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K2" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Bodily injury per accident</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>$50,000</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code Section 9-25-4-5</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code 9-25-4-5 - Financial Responsibility Minimum Limits</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-9-motor-vehicles/in-code-sect-9-25-4-5.html</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J3" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K3" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Minimum liability</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Property damage</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>$25,000 (raised from $10,000, effective July 1, 2018)</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code Section 9-25-4-5</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code 9-25-4-5 - Financial Responsibility Minimum Limits</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-9-motor-vehicles/in-code-sect-9-25-4-5.html</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Uninsured/underinsured motorist coverage</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Insurers must make UM/UIM coverage available at limits at least equal to the policy's bodily injury liability limits; underinsured motorist coverage may never be sold below $50,000</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code Section 27-7-5-2</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code 27-7-5-2 - Uninsured/Underinsured Motorist Coverage</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-27-insurance/in-code-sect-27-7-5-2.html</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>UM/UIM rejection rules</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>A named insured may reject UM and UIM coverage together, or reject either one separately if the insurer offers the other separately; the rejection must identify which coverage is rejected and its effective date, binds every other person insured under the policy, and the insurer need not re-offer the coverage on renewal or replacement policies unless the insured later requests it in writing</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code Section 27-7-5-2</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Indiana Code 27-7-5-2 - Uninsured/Underinsured Motorist Coverage</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-27-insurance/in-code-sect-27-7-5-2.html</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="B1" s="28" t="inlineStr">
+        <is>
+          <t>Fact</t>
+        </is>
+      </c>
+      <c r="C1" s="28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D1" s="28" t="inlineStr">
+        <is>
+          <t>Legal Citation</t>
+        </is>
+      </c>
+      <c r="E1" s="28" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="28" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="G1" s="28" t="inlineStr">
+        <is>
+          <t>Date Collected</t>
+        </is>
+      </c>
+      <c r="H1" s="28" t="inlineStr">
+        <is>
+          <t>Geographic Scope</t>
+        </is>
+      </c>
+      <c r="I1" s="28" t="inlineStr">
+        <is>
+          <t>Data Type</t>
+        </is>
+      </c>
+      <c r="J1" s="28" t="inlineStr">
+        <is>
+          <t>Verification Status</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="L1" s="28" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B2" s="28" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C2" s="28" t="inlineStr">
+        <is>
+          <t>The Indiana Basic Property Insurance Underwriting Association (the Indiana FAIR Plan) was established October 28, 1968 to provide property insurance to applicants unable to obtain coverage in the standard market; it is a last-resort option, not a competing alternative</t>
+        </is>
+      </c>
+      <c r="D2" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E2" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (Indiana Basic Property Insurance Underwriting Association)</t>
+        </is>
+      </c>
+      <c r="F2" s="28" t="inlineStr">
+        <is>
+          <t>https://www.indianafairplan.com</t>
+        </is>
+      </c>
+      <c r="G2" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H2" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I2" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J2" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K2" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B3" s="28" t="inlineStr">
+        <is>
+          <t>Eligibility</t>
+        </is>
+      </c>
+      <c r="C3" s="28" t="inlineStr">
+        <is>
+          <t>Applicants must have been declined coverage by at least three non-related insurance companies, which is verified during the application process</t>
+        </is>
+      </c>
+      <c r="D3" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E3" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (Indiana Basic Property Insurance Underwriting Association)</t>
+        </is>
+      </c>
+      <c r="F3" s="28" t="inlineStr">
+        <is>
+          <t>https://www.indianafairplan.com</t>
+        </is>
+      </c>
+      <c r="G3" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H3" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I3" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J3" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K3" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Coverage provided</t>
+        </is>
+      </c>
+      <c r="C4" s="28" t="inlineStr">
+        <is>
+          <t>Dwelling insurance and commercial property insurance</t>
+        </is>
+      </c>
+      <c r="D4" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E4" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (Indiana Basic Property Insurance Underwriting Association)</t>
+        </is>
+      </c>
+      <c r="F4" s="28" t="inlineStr">
+        <is>
+          <t>https://www.indianafairplan.com</t>
+        </is>
+      </c>
+      <c r="G4" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H4" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I4" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J4" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K4" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Coverage limits</t>
+        </is>
+      </c>
+      <c r="C5" s="28" t="inlineStr">
+        <is>
+          <t>Dwellings are capped at a combined $250,000 for building and contents; commercial property is capped at a combined $1,000,000 for building and contents</t>
+        </is>
+      </c>
+      <c r="D5" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (Indiana Basic Property Insurance Underwriting Association)</t>
+        </is>
+      </c>
+      <c r="F5" s="28" t="inlineStr">
+        <is>
+          <t>https://www.indianafairplan.com</t>
+        </is>
+      </c>
+      <c r="G5" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H5" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I5" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J5" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K5" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Contact</t>
+        </is>
+      </c>
+      <c r="C6" s="28" t="inlineStr">
+        <is>
+          <t>3502 Woodview Trace, Suite 100, Indianapolis, IN 46268; claims 317-692-0572, member questions 317-692-0578, agent/agency access and all other questions 317-692-0559; Monday-Thursday 7:00 AM-4:00 PM, Friday 7:30 AM-11:30 AM (appointment required for visits)</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (plan administrator)</t>
+        </is>
+      </c>
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Indiana FAIR Plan (Indiana Basic Property Insurance Underwriting Association)</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="inlineStr">
+        <is>
+          <t>https://www.indianafairplan.com</t>
+        </is>
+      </c>
+      <c r="G6" s="48" t="n">
+        <v>46296</v>
+      </c>
+      <c r="H6" s="28" t="inlineStr">
+        <is>
+          <t>Indiana</t>
+        </is>
+      </c>
+      <c r="I6" s="28" t="inlineStr">
+        <is>
+          <t>Regulator-published</t>
+        </is>
+      </c>
+      <c r="J6" s="28" t="inlineStr">
+        <is>
+          <t>Primary source</t>
+        </is>
+      </c>
+      <c r="K6" s="48" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
@@ -36905,17 +37742,39 @@
           <t>Indiana</t>
         </is>
       </c>
-      <c r="B16" s="41" t="n"/>
-      <c r="C16" s="41" t="n"/>
-      <c r="D16" s="41" t="n"/>
+      <c r="B16" s="41" t="n">
+        <v>25</v>
+      </c>
+      <c r="C16" s="41" t="n">
+        <v>50</v>
+      </c>
+      <c r="D16" s="41" t="n">
+        <v>25</v>
+      </c>
       <c r="E16" s="41" t="n"/>
       <c r="F16" s="41" t="n"/>
-      <c r="G16" s="41" t="n"/>
-      <c r="H16" s="41" t="n"/>
-      <c r="I16" s="41" t="n"/>
-      <c r="J16" s="42" t="n"/>
+      <c r="G16" s="41" t="inlineStr">
+        <is>
+          <t>UM/UIM available; UIM cannot be sold below $50,000</t>
+        </is>
+      </c>
+      <c r="H16" s="41" t="inlineStr">
+        <is>
+          <t>Property damage raised from $10,000, effective July 1, 2018</t>
+        </is>
+      </c>
+      <c r="I16" s="41" t="inlineStr">
+        <is>
+          <t>Indiana Code 9-25-4-5 - Financial Responsibility Minimum Limits</t>
+        </is>
+      </c>
+      <c r="J16" s="42" t="inlineStr">
+        <is>
+          <t>https://codes.findlaw.com/in/title-9-motor-vehicles/in-code-sect-9-25-4-5.html</t>
+        </is>
+      </c>
       <c r="K16" s="43" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="L16" s="41" t="inlineStr">
         <is>
@@ -36924,16 +37783,16 @@
       </c>
       <c r="M16" s="41" t="inlineStr">
         <is>
-          <t>Placeholder</t>
+          <t>Regulator-published</t>
         </is>
       </c>
       <c r="N16" s="47" t="inlineStr">
         <is>
-          <t>Not researched</t>
+          <t>Primary source</t>
         </is>
       </c>
       <c r="O16" s="43" t="n">
-        <v>46295</v>
+        <v>46296</v>
       </c>
       <c r="P16" s="41" t="inlineStr">
         <is>

</xml_diff>